<commit_message>
Generic app for the App Store: no club names, blank defaults, sample club with example names; store texts, manual, privacy policy; selection bar above the tab bar; draft-only App Store listing workflow
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019Zy7EWLw516wT4YZykUHCa
</commit_message>
<xml_diff>
--- a/Tests/ClubCoreTests/Fixtures/members.xlsx
+++ b/Tests/ClubCoreTests/Fixtures/members.xlsx
@@ -449,17 +449,17 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Bojan</t>
+          <t>Ivan</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Šurbatović</t>
+          <t>Šimić</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>bojan@example.com</t>
+          <t>ivan@example.com</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>

</xml_diff>